<commit_message>
F&D: mark all 6 PO questions ANSWERED (Milos 2026-07-09) in PO-Questions-SIMPLE
- Each question now shows Milos's answer + one-sentence resulting action
- Internal QA map gains a 'PO answer -> outcome' column
- gen_po_questions_simple.py updated (answer/action baked in); xlsx regenerated

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/fees-discounts/PO-Questions-SIMPLE.xlsx
+++ b/build/fees-discounts/PO-Questions-SIMPLE.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -479,20 +479,20 @@
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="2" t="inlineStr"/>
     </row>
-    <row r="3" ht="15" customHeight="1">
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This is about the new Fees &amp; Discounts feature.</t>
+          <t>STATUS: ALL 6 QUESTIONS ANSWERED (Milos, received 2026-07-09). Thank you!</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="inlineStr"/>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="15" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>While checking it over, we found a handful of spots where the app behaves a little differently than the original write-up described. None of these are problems on their own - we just want your quick call on each one so we know which way you'd like it to work.</t>
+          <t>This is about the new Fees &amp; Discounts feature.</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,27 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>There are no wrong answers. On the "PO Questions" tab, each row has a short description of what happens now, the question, and simple A/B options. Please pick an option (or write your own) in the "Your answer" column.</t>
+          <t>While checking it over, we found a handful of spots where the app behaves a little differently than the original write-up described. None of these are problems on their own - we just wanted your quick call on each one so we know which way you'd like it to work.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="inlineStr"/>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>It should take just a few minutes. Thank you!</t>
+          <t>The "PO Questions" tab now shows each question with the answer received in the "Your answer" column and what we are doing about it in the "Resulting action" column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Thank you - your answers are helping us finish this feature the way you want it.</t>
         </is>
       </c>
     </row>
@@ -527,15 +537,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -569,6 +580,11 @@
           <t>Your answer</t>
         </is>
       </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Resulting action</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="110" customHeight="1">
       <c r="A2" s="4" t="n">
@@ -595,7 +611,16 @@
 B) Change it so each fee and discount is listed on its own row.</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr"/>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>ANSWERED - B. "This is actually a story defect. It was fixed originally in Branko's design, but appears to have regressed in the spec."</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>The row-by-row list is what's intended, so the current combined total is a defect and a dev ticket has been drafted to fix it.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="110" customHeight="1">
       <c r="A3" s="4" t="n">
@@ -622,7 +647,16 @@
 B) No - it should behave differently (please describe).</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>ANSWERED - A. Adding it only once is correct; treat as settled.</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>This is settled - the earlier double-add worry is closed and our test cases will be updated to expect exactly one added fee.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="110" customHeight="1">
       <c r="A4" s="4" t="n">
@@ -649,7 +683,16 @@
 B) It should be part of this release - the visible option needs to be added.</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>ANSWERED - B. It should be part of this release - the visible option needs to be added.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>The missing Processing Fee option is an in-scope gap for this release, so a dev ticket has been drafted to add it and our Processing Fee test cases stay in scope.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="110" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -676,7 +719,16 @@
 B) Change it so the button is greyed out until the form is filled in correctly.</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>ANSWERED - B. Change it so the button is greyed out until the form is filled in correctly.</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>The always-clickable button is a defect, so a dev ticket has been drafted to keep the button greyed out until the form is valid.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="110" customHeight="1">
       <c r="A6" s="4" t="n">
@@ -703,7 +755,16 @@
 B) Change it so extra ones collapse under a "show more" option.</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>ANSWERED - B. "Similar to #1. It was fixed in the design with a 'show more' ... apparently I didn't define this properly in the spec."</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>The "show more" collapse is what's intended, so its absence is a defect and a dev ticket has been drafted to add it.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="110" customHeight="1">
       <c r="A7" s="4" t="n">
@@ -730,7 +791,16 @@
 B) Change it so you can tick several and add them all at once.</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>ANSWERED - A. Keep as-is - "judgement call. There's higher risk that a user will inadvertently add multiples ... the additional clicks are worthwhile."</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>One-at-a-time is accepted as the intended behavior - no bug will be filed and our test cases will be reworded to match it.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -743,12 +813,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -774,6 +845,11 @@
           <t>Cases / refs covered</t>
         </is>
       </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>PO answer -&gt; outcome</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -791,6 +867,11 @@
           <t>FD-STATS-001 (BUG-FD-2 / FDBUG-6); also settles FD-STATS-002, FD-STATS-004</t>
         </is>
       </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>B -&gt; confirmed DEFECT (per-row regressed from Branko's design); dev ticket drafted (jira-bug-drafts.md TICKET 8); keep spec expected</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -808,6 +889,11 @@
           <t>FD-CUST-016 / FD-VAL-007 (BUG-FD-1 double-add; did not reproduce - confirm S9 dedupe shipped)</t>
         </is>
       </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>A -&gt; settled; close BUG-FD-1; re-scope EXPECTED to exactly-one adjustment</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -825,6 +911,11 @@
           <t>NOTE-FD-4 (Story 8 Processing Fee - backend accepts it, builder UI missing)</t>
         </is>
       </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>B -&gt; in-scope build GAP; dev ticket drafted (TICKET 11); FD-PROC-* stay v1</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -842,6 +933,11 @@
           <t>FD-WO-005 / FD-VAL-001 (BUG-FD-4 - confirm button enabled; validation on submit)</t>
         </is>
       </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>B -&gt; confirmed DEFECT (disabled-until-valid); dev ticket drafted (TICKET 9); keep spec expected</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -859,6 +955,11 @@
           <t>FD-INLINE-003 (BUG-FD-5 - no "Show N more" collapse on line adjustments)</t>
         </is>
       </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>B -&gt; confirmed DEFECT (show-more was in design); dev ticket drafted (TICKET 10); keep spec expected</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -876,18 +977,23 @@
           <t>FD-CUST-005 (NOTE-FD-5 / FDBUG-7); ruling also settles FD-CUST-003/004/006/007</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>A -&gt; ACCEPTED behavior; close FDBUG-7 won't-fix; adopt single-select case-wording updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Note: Two threads were REMOVED from the PO document as dev bugs (not product decisions), already covered in jira-bug-drafts.md: the whole-WO permission "hidden but not backend-enforced" item (BUG-FD-3), and the customer total/estimate leaving out the fee/discount amount (FDBUG-1). Pure code-bug tickets and the Part 2 case-update wording proposals are also excluded. Source: build/fees-discounts/Deviations-and-Questions-for-PO.md</t>
+          <t>Note: Answers received 2026-07-09 via the PO answer sheet, archived as data-sheet-source.xlsx/.csv/.md; verbatim answers + outcomes in spec-v1-reconciliation.md sec.3. Two threads were REMOVED from the PO document as dev bugs (not product decisions), already covered in jira-bug-drafts.md: the whole-WO permission "hidden but not backend-enforced" item (BUG-FD-3, still open with dev), and the customer total/estimate leaving out the fee/discount amount (FDBUG-1, on hold pending a US-tax re-check). Pure code-bug tickets and the Part 2 case-update wording proposals are also excluded. Source: build/fees-discounts/Deviations-and-Questions-for-PO.md</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>